<commit_message>
skill báo cáo tháng nâng cấp
</commit_message>
<xml_diff>
--- a/van_ban_du_thao/2026/Quyet_dinh/Phu_luc_nhiem_vu_CDS_QD11_va_KH04.xlsx
+++ b/van_ban_du_thao/2026/Quyet_dinh/Phu_luc_nhiem_vu_CDS_QD11_va_KH04.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Chuyên viên ảo\van_ban_du_thao\2026\Quyet_dinh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC7C6BD-10BF-4D9D-B4FE-3275A9AB0DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36928195-4A7B-485D-B045-4025E45B68B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh_muc" sheetId="1" state="hidden" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="247">
   <si>
     <t>Mã số</t>
   </si>
@@ -439,12 +439,6 @@
     <t>Trung tâm Hành chính công</t>
   </si>
   <si>
-    <t>PHỤ LỤC: DANH MỤC NHIỆM VỤ TRỌNG TÂM TRIỂN KHAI THEO KẾ HOẠCH SỐ 04-KH/ĐU</t>
-  </si>
-  <si>
-    <t>(Ban hành kèm theo Kế hoạch số 04-KH/ĐU ngày 10/7/2026 của Đảng uỷ xã Công Hải)</t>
-  </si>
-  <si>
     <t>STT</t>
   </si>
   <si>
@@ -802,14 +796,55 @@
     <t>Cơ quan chủ trì</t>
   </si>
   <si>
-    <t>PHỤ LỤC: DANH MỤC CÔNG VIỆC CHUYỂN ĐỔI SỐ QUÝ IV/2026</t>
+    <r>
+      <t>PHỤ LỤC II
+DANH MỤC NHIỆM VỤ TRỌNG TÂM 100 NGÀY THÁO GỠ ĐIỂM NGHẼN CHUYỂN ĐỔI SỐ</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(Ban hành kèm theo Quyết định số 171-QĐ/ĐU ngày 29/10/2026 của Ban Thường vụ Đảng uỷ)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHỤ LỤC I
+DANH MỤC NHIỆM VỤ TRỌNG CHUYỂN ĐỔI SỐ QUÝ IV/2026
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(Ban hành kèm theo Quyết định số 171-QĐ/ĐU ngày 29/10/2026 của Ban Thường vụ Đảng uỷ)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -819,18 +854,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF333333"/>
       <name val="Times New Roman"/>
     </font>
     <font>
@@ -855,6 +878,27 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -936,43 +980,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1341,16 +1382,16 @@
     <col min="7" max="7" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+    <row r="1" spans="1:7" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="3" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -1363,7 +1404,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>4</v>
@@ -1376,22 +1417,22 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
     </row>
     <row r="5" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C5" s="3">
         <v>3</v>
@@ -1502,15 +1543,15 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
     </row>
     <row r="11" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -1526,7 +1567,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>36</v>
@@ -1549,7 +1590,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>36</v>
@@ -1572,7 +1613,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>42</v>
@@ -1685,7 +1726,7 @@
         <v>9</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>63</v>
@@ -1708,7 +1749,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>67</v>
@@ -1731,7 +1772,7 @@
         <v>71</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>72</v>
@@ -1787,15 +1828,15 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
@@ -1959,15 +2000,15 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
     </row>
     <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
@@ -2091,7 +2132,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2101,679 +2142,669 @@
     <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="3" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="B3" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-    </row>
-    <row r="4" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="2" t="s">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="C5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="D8" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-    </row>
-    <row r="9" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C9" s="8" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="D19" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="C12" s="5" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+    </row>
+    <row r="24" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="7" t="s">
+      <c r="D24" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-    </row>
-    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>245</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-    </row>
-    <row r="20" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C20" s="5" t="s">
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-    </row>
-    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="C25" s="8" t="s">
+      <c r="D27" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="D28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+    </row>
+    <row r="31" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+    </row>
+    <row r="36" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+    </row>
+    <row r="39" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="D39" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+    </row>
+    <row r="41" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-    </row>
-    <row r="32" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C34" s="5" t="s">
+      <c r="D41" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-    </row>
-    <row r="37" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-    </row>
-    <row r="40" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
-        <v>224</v>
-      </c>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-    </row>
-    <row r="42" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+      <c r="D44" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="E44" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="C45" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>237</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A14:E14"/>
+  <mergeCells count="10">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="94" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2784,7 +2815,7 @@
           <x14:formula1>
             <xm:f>Danh_muc!$A$1:$A$8</xm:f>
           </x14:formula1>
-          <xm:sqref>C6 C7 C9 C10 C11 C12 C13 C15 C16 C17 C18 C20 C21 C22 C23 C25 C26 C27 C28 C29 C30 C32 C33 C34 C35 C37 C38 C40 C42 C43 C44 C45</xm:sqref>
+          <xm:sqref>C5 C6 C8 C9 C10 C11 C12 C14 C15 C16 C17 C19 C20 C21 C22 C24 C25 C26 C27 C28 C29 C31 C32 C33 C34 C36 C37 C39 C41 C42 C43 C44</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>